<commit_message>
Added more contents and playlists
</commit_message>
<xml_diff>
--- a/Atlas_Library.xlsx
+++ b/Atlas_Library.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cyril\Documents\antigravity\elegant-pasteur\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3454A8BB-36A2-45C6-99C3-FB84D8A9A0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DBFE18-98CA-4203-990D-336318E26AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2974379D-9C44-4FFD-B212-20BC61C97767}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
   <si>
     <t>Title</t>
   </si>
@@ -50,24 +50,9 @@
     <t>Active</t>
   </si>
   <si>
-    <t>Professional Ethics English Revision</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=47YW5sWmb8Y</t>
-  </si>
-  <si>
     <t>General</t>
   </si>
   <si>
-    <t>YouTube</t>
-  </si>
-  <si>
-    <t>CA Shubham Keswani English Revision</t>
-  </si>
-  <si>
-    <t>revision,ethics</t>
-  </si>
-  <si>
     <t>ICAI Official Website</t>
   </si>
   <si>
@@ -86,21 +71,9 @@
     <t>icai,official</t>
   </si>
   <si>
-    <t>RTP</t>
-  </si>
-  <si>
-    <t>Final RTP for May 2026</t>
-  </si>
-  <si>
-    <t>rtp,fr,final</t>
-  </si>
-  <si>
     <t>AFM</t>
   </si>
   <si>
-    <t>https://resource.cdn.icai.org/91030bos-aps4369-final-may2026-p2.pdf</t>
-  </si>
-  <si>
     <t>https://boslive.icai.org/</t>
   </si>
   <si>
@@ -119,10 +92,70 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>1.0.1</t>
-  </si>
-  <si>
-    <t>Initial Atlas Library with sample resources-Test</t>
+    <t>1.0.2</t>
+  </si>
+  <si>
+    <t>Initial Atlas Library with sample resources-Test2</t>
+  </si>
+  <si>
+    <t>BOS Knowledge Portal -ICAI</t>
+  </si>
+  <si>
+    <t>BOS Knowledge Portal</t>
+  </si>
+  <si>
+    <t>https://youtube.com/playlist?list=PLZg_w2bN180b-fzkn1GIOau71UnPzyxGd&amp;si=qzLU_huwlohltByz</t>
+  </si>
+  <si>
+    <t>AFM Revision Playlist-Bhavik Chokshi</t>
+  </si>
+  <si>
+    <t>Audit</t>
+  </si>
+  <si>
+    <t>https://youtube.com/playlist?list=PLjURe7lJQG-ovHBiKStSvekRcvv6csYR_&amp;si=ghOE67lhrc4YGR3P</t>
+  </si>
+  <si>
+    <t>Audit Revision Playlist- Shubham Keswani</t>
+  </si>
+  <si>
+    <t>Youtube</t>
+  </si>
+  <si>
+    <t>AFM English Revision Playlist</t>
+  </si>
+  <si>
+    <t>Audit-English Revision Playlist-SK</t>
+  </si>
+  <si>
+    <t>FR Revision Playlist-Bhavik Chokshi</t>
+  </si>
+  <si>
+    <t>https://youtube.com/playlist?list=PLZg_w2bN180b5AFUAWFRYtibGzhIt-E_p&amp;si=BOpEXZ-W9RjqbBAJ</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>FR English Revision Playlist-Bhavik Chokshi</t>
+  </si>
+  <si>
+    <t>https://youtube.com/playlist?list=PLm8RLlq6Pj_lQV6xwy8JdVIElHAa81bAJ&amp;si=Z0HXjgMHpfEhS5XA</t>
+  </si>
+  <si>
+    <t>FR Revision Playlist-Aakash Kandoi</t>
+  </si>
+  <si>
+    <t>FR English Revision Playlist-Aakash Kandoi</t>
+  </si>
+  <si>
+    <t>https://youtu.be/wx68ZCCOTnc?si=fBYepsKROdrsm1KI</t>
+  </si>
+  <si>
+    <t>Auditing Marathon-Ram Harsha</t>
+  </si>
+  <si>
+    <t>Auditing Marathon-Ram Harsha-11hrs</t>
   </si>
 </sst>
 </file>
@@ -955,23 +988,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1">
         <v>46205</v>
@@ -979,10 +1012,10 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -992,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D328AF79-2E8E-46C3-A800-BD98BF932E6F}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
@@ -1037,28 +1070,28 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="b">
         <v>1</v>
@@ -1066,65 +1099,122 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3" t="b">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated with more playlist files+thumbnails
</commit_message>
<xml_diff>
--- a/Atlas_Library.xlsx
+++ b/Atlas_Library.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cyril\Documents\antigravity\elegant-pasteur\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C21D1C-7EB0-45A8-A9B1-270FCD99B1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FE6BB6-79AC-4FCE-8BB8-68DB56B3E0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2974379D-9C44-4FFD-B212-20BC61C97767}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2974379D-9C44-4FFD-B212-20BC61C97767}"/>
   </bookViews>
   <sheets>
     <sheet name="Atlas_Library_Version" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
   <si>
     <t>Title</t>
   </si>
@@ -56,9 +56,6 @@
     <t>ICAI Official Website</t>
   </si>
   <si>
-    <t>https://www.icai.org</t>
-  </si>
-  <si>
     <t>Website</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>1.0.2</t>
-  </si>
-  <si>
     <t>Initial Atlas Library with sample resources-Test2</t>
   </si>
   <si>
@@ -101,18 +95,12 @@
     <t>BOS Knowledge Portal</t>
   </si>
   <si>
-    <t>https://youtube.com/playlist?list=PLZg_w2bN180b-fzkn1GIOau71UnPzyxGd&amp;si=qzLU_huwlohltByz</t>
-  </si>
-  <si>
     <t>AFM Revision Playlist-Bhavik Chokshi</t>
   </si>
   <si>
     <t>Audit</t>
   </si>
   <si>
-    <t>https://youtube.com/playlist?list=PLjURe7lJQG-ovHBiKStSvekRcvv6csYR_&amp;si=ghOE67lhrc4YGR3P</t>
-  </si>
-  <si>
     <t>Audit Revision Playlist- Shubham Keswani</t>
   </si>
   <si>
@@ -128,18 +116,12 @@
     <t>FR Revision Playlist-Bhavik Chokshi</t>
   </si>
   <si>
-    <t>https://youtube.com/playlist?list=PLZg_w2bN180b5AFUAWFRYtibGzhIt-E_p&amp;si=BOpEXZ-W9RjqbBAJ</t>
-  </si>
-  <si>
     <t>FR</t>
   </si>
   <si>
     <t>FR English Revision Playlist-Bhavik Chokshi</t>
   </si>
   <si>
-    <t>https://youtube.com/playlist?list=PLm8RLlq6Pj_lQV6xwy8JdVIElHAa81bAJ&amp;si=Z0HXjgMHpfEhS5XA</t>
-  </si>
-  <si>
     <t>FR Revision Playlist-Aakash Kandoi</t>
   </si>
   <si>
@@ -153,6 +135,27 @@
   </si>
   <si>
     <t>Auditing Marathon-Ram Harsha-11hrs</t>
+  </si>
+  <si>
+    <t>1.0.3</t>
+  </si>
+  <si>
+    <t>https://youtu.be/N2tOhF0bpTo?si=9JlRyLZHUrhBM07_</t>
+  </si>
+  <si>
+    <t>https://youtu.be/daZzaYYPfkk?si=jxAReFlEpiGvFkTa</t>
+  </si>
+  <si>
+    <t>https://youtu.be/VuhkMYOjQmA?si=0wHCoX1FxhSzPflO</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bxdpiOEGUQ0?si=OTxWVw1CSCfs7HeF</t>
+  </si>
+  <si>
+    <t>https://youtube.com/playlist?list=PL_zH8wj_XM2uLCpNYhwOKkMcsMvgjq6ES&amp;si=VHPy8ierZM6N35cP</t>
+  </si>
+  <si>
+    <t>AFM Marathon-Tabish Hassan</t>
   </si>
 </sst>
 </file>
@@ -985,23 +988,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
         <v>17</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1">
         <v>46205</v>
@@ -1009,10 +1012,10 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1022,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D328AF79-2E8E-46C3-A800-BD98BF932E6F}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
@@ -1070,139 +1073,159 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
       <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
       </c>
       <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="B4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
         <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
         <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edited icai address and afm
</commit_message>
<xml_diff>
--- a/Atlas_Library.xlsx
+++ b/Atlas_Library.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cyril\Documents\antigravity\elegant-pasteur\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FE6BB6-79AC-4FCE-8BB8-68DB56B3E0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8BBB27-46B3-4569-8882-A750DBD3A37A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2974379D-9C44-4FFD-B212-20BC61C97767}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2974379D-9C44-4FFD-B212-20BC61C97767}"/>
   </bookViews>
   <sheets>
     <sheet name="Atlas_Library_Version" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t>Title</t>
   </si>
@@ -86,9 +86,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Initial Atlas Library with sample resources-Test2</t>
-  </si>
-  <si>
     <t>BOS Knowledge Portal -ICAI</t>
   </si>
   <si>
@@ -137,9 +134,6 @@
     <t>Auditing Marathon-Ram Harsha-11hrs</t>
   </si>
   <si>
-    <t>1.0.3</t>
-  </si>
-  <si>
     <t>https://youtu.be/N2tOhF0bpTo?si=9JlRyLZHUrhBM07_</t>
   </si>
   <si>
@@ -152,10 +146,19 @@
     <t>https://youtu.be/bxdpiOEGUQ0?si=OTxWVw1CSCfs7HeF</t>
   </si>
   <si>
-    <t>https://youtube.com/playlist?list=PL_zH8wj_XM2uLCpNYhwOKkMcsMvgjq6ES&amp;si=VHPy8ierZM6N35cP</t>
-  </si>
-  <si>
     <t>AFM Marathon-Tabish Hassan</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/live/wI91DJOytDk?si=MPgfmNSLH8cphEVc</t>
+  </si>
+  <si>
+    <t>https://icai.org/</t>
+  </si>
+  <si>
+    <t>1.0.4</t>
+  </si>
+  <si>
+    <t>Initial Atlas Library with sample resources-Test3</t>
   </si>
 </sst>
 </file>
@@ -999,7 +1002,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1007,7 +1010,7 @@
         <v>19</v>
       </c>
       <c r="B3" s="1">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1015,7 +1018,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1073,7 +1076,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -1090,7 +1093,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -1105,127 +1108,127 @@
         <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
       </c>
       <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
         <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
         <v>30</v>
       </c>
-      <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
         <v>31</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
         <v>33</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" t="s">
         <v>36</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>